<commit_message>
[FEAT]: improve pipeline visualization by encapsulating components in a metanode
</commit_message>
<xml_diff>
--- a/data/logs/ean-problems/logs.xlsx
+++ b/data/logs/ean-problems/logs.xlsx
@@ -56,7 +56,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -181,46 +181,6 @@
         <v>120.0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr" s="0">
-        <is>
-          <t>8410500028794</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr" s="0">
-        <is>
-          <t>440</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr" s="0">
-        <is>
-          <t>leche</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr" s="0">
-        <is>
-          <t>Yogures estilo griego, Yogures naturales</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr" s="0">
-        <is>
-          <t>https://images.openfoodfacts.org/images/products/841/050/002/8794/front_es.35.400.jpg</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr" s="0">
-        <is>
-          <t>Griego natural</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr" s="0">
-        <is>
-          <t>29/10/2026</t>
-        </is>
-      </c>
-      <c r="H4" t="n" s="0">
-        <v>4.0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="portrait" paperSize="9"/>
@@ -229,7 +189,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -240,22 +200,29 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>expirationdate</t>
+          <t>pipeline_stage</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>quantity</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>pipeline_stage</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>failure_reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>8410500028794</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Product Matching</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>EAN not found in CSV</t>
         </is>
       </c>
     </row>

</xml_diff>